<commit_message>
update pembaharuan timesheet bmp
</commit_message>
<xml_diff>
--- a/1_Data_Master/Data Absensi_BMP.xlsx
+++ b/1_Data_Master/Data Absensi_BMP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GENERAL PSD\PENDINGAN LINDAA 2026\GENERAL 2026\00. PORTAL TIMESHEET\1_Data_Master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C81FC8-3603-4A84-869A-EF8AD25A25C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8755AFA0-72A9-4351-8673-ABA1F8973DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CEF79333-F3A4-451D-BE26-4BA9C1711C1C}"/>
   </bookViews>
@@ -1322,12 +1322,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1347,6 +1341,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2899,7 +2899,8 @@
     <col min="6" max="6" width="48.7265625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24" style="1" customWidth="1"/>
     <col min="8" max="8" width="14.453125" style="1" customWidth="1"/>
-    <col min="9" max="38" width="5.7265625" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="38" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="20.453125" customWidth="1"/>
     <col min="40" max="40" width="24.90625" customWidth="1"/>
     <col min="41" max="41" width="33.54296875" customWidth="1"/>
@@ -2930,123 +2931,124 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="97">
-        <v>1</v>
-      </c>
-      <c r="J1" s="97">
+      <c r="I1" s="104">
+        <v>46266</v>
+      </c>
+      <c r="J1" s="104">
         <f>I1+1</f>
-        <v>2</v>
-      </c>
-      <c r="K1" s="97">
+        <v>46267</v>
+      </c>
+      <c r="K1" s="104">
         <f t="shared" ref="K1:AK1" si="0">J1+1</f>
-        <v>3</v>
-      </c>
-      <c r="L1" s="97">
+        <v>46268</v>
+      </c>
+      <c r="L1" s="104">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="M1" s="97">
+        <v>46269</v>
+      </c>
+      <c r="M1" s="104">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="N1" s="97">
+        <v>46270</v>
+      </c>
+      <c r="N1" s="104">
         <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="O1" s="97">
+        <v>46271</v>
+      </c>
+      <c r="O1" s="104">
         <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="P1" s="97">
+        <v>46272</v>
+      </c>
+      <c r="P1" s="104">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="Q1" s="97">
+        <v>46273</v>
+      </c>
+      <c r="Q1" s="104">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="R1" s="97">
+        <v>46274</v>
+      </c>
+      <c r="R1" s="104">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="S1" s="97">
+        <v>46275</v>
+      </c>
+      <c r="S1" s="104">
         <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-      <c r="T1" s="97">
+        <v>46276</v>
+      </c>
+      <c r="T1" s="104">
         <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="U1" s="97">
+        <v>46277</v>
+      </c>
+      <c r="U1" s="104">
         <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="V1" s="97">
+        <v>46278</v>
+      </c>
+      <c r="V1" s="104">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="W1" s="97">
+        <v>46279</v>
+      </c>
+      <c r="W1" s="104">
         <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="X1" s="97">
+        <v>46280</v>
+      </c>
+      <c r="X1" s="104">
         <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="Y1" s="98">
+        <v>46281</v>
+      </c>
+      <c r="Y1" s="105">
         <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="Z1" s="97">
+        <v>46282</v>
+      </c>
+      <c r="Z1" s="104">
         <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="AA1" s="97">
+        <v>46283</v>
+      </c>
+      <c r="AA1" s="104">
         <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="AB1" s="97">
+        <v>46284</v>
+      </c>
+      <c r="AB1" s="104">
         <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="AC1" s="97">
+        <v>46285</v>
+      </c>
+      <c r="AC1" s="104">
         <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="AD1" s="97">
+        <v>46286</v>
+      </c>
+      <c r="AD1" s="104">
         <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="AE1" s="97">
+        <v>46287</v>
+      </c>
+      <c r="AE1" s="104">
         <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="AF1" s="97">
+        <v>46288</v>
+      </c>
+      <c r="AF1" s="104">
         <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="AG1" s="97">
+        <v>46289</v>
+      </c>
+      <c r="AG1" s="104">
         <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="AH1" s="97">
+        <v>46290</v>
+      </c>
+      <c r="AH1" s="104">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="AI1" s="97">
+        <v>46291</v>
+      </c>
+      <c r="AI1" s="104">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="AJ1" s="97">
+        <v>46292</v>
+      </c>
+      <c r="AJ1" s="104">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="AK1" s="97">
+        <v>46293</v>
+      </c>
+      <c r="AK1" s="104">
         <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="AL1" s="97">
-        <v>30</v>
+        <v>46294</v>
+      </c>
+      <c r="AL1" s="104">
+        <f>AK1+1</f>
+        <v>46295</v>
       </c>
       <c r="AO1" s="3" t="s">
         <v>4</v>
@@ -8428,10 +8430,10 @@
       <c r="R47" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="S47" s="105" t="s">
-        <v>22</v>
-      </c>
-      <c r="T47" s="105" t="s">
+      <c r="S47" s="103" t="s">
+        <v>22</v>
+      </c>
+      <c r="T47" s="103" t="s">
         <v>15</v>
       </c>
       <c r="U47" s="18" t="s">
@@ -8543,10 +8545,10 @@
       <c r="R48" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="S48" s="105" t="s">
-        <v>22</v>
-      </c>
-      <c r="T48" s="105" t="s">
+      <c r="S48" s="103" t="s">
+        <v>22</v>
+      </c>
+      <c r="T48" s="103" t="s">
         <v>22</v>
       </c>
       <c r="U48" s="18" t="s">
@@ -8658,10 +8660,10 @@
       <c r="R49" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="S49" s="105" t="s">
-        <v>0</v>
-      </c>
-      <c r="T49" s="105" t="s">
+      <c r="S49" s="103" t="s">
+        <v>0</v>
+      </c>
+      <c r="T49" s="103" t="s">
         <v>0</v>
       </c>
       <c r="U49" s="18" t="s">
@@ -8773,7 +8775,7 @@
       <c r="R50" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S50" s="105" t="s">
+      <c r="S50" s="103" t="s">
         <v>0</v>
       </c>
       <c r="T50" s="7" t="s">
@@ -15824,7 +15826,7 @@
       <c r="C3" s="65">
         <v>207231</v>
       </c>
-      <c r="D3" s="104" t="s">
+      <c r="D3" s="102" t="s">
         <v>98</v>
       </c>
       <c r="E3" s="67">
@@ -16104,7 +16106,7 @@
       <c r="C10" s="65">
         <v>207231</v>
       </c>
-      <c r="D10" s="104" t="s">
+      <c r="D10" s="102" t="s">
         <v>98</v>
       </c>
       <c r="E10" s="67">
@@ -16182,8 +16184,8 @@
         <v>13</v>
       </c>
       <c r="C12" s="65"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="103"/>
+      <c r="D12" s="97"/>
+      <c r="E12" s="101"/>
       <c r="F12" s="64"/>
       <c r="G12" s="68"/>
       <c r="H12" s="69"/>
@@ -16191,9 +16193,9 @@
       <c r="J12" s="64"/>
       <c r="K12" s="64"/>
       <c r="L12" s="71"/>
-      <c r="M12" s="100"/>
-      <c r="N12" s="100"/>
-      <c r="O12" s="101"/>
+      <c r="M12" s="98"/>
+      <c r="N12" s="98"/>
+      <c r="O12" s="99"/>
       <c r="P12" s="72"/>
       <c r="Q12" s="73"/>
     </row>
@@ -16206,8 +16208,8 @@
         <v>14</v>
       </c>
       <c r="C13" s="65"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="103"/>
+      <c r="D13" s="97"/>
+      <c r="E13" s="101"/>
       <c r="F13" s="64"/>
       <c r="G13" s="68"/>
       <c r="H13" s="69"/>
@@ -16215,9 +16217,9 @@
       <c r="J13" s="64"/>
       <c r="K13" s="64"/>
       <c r="L13" s="71"/>
-      <c r="M13" s="100"/>
-      <c r="N13" s="100"/>
-      <c r="O13" s="101"/>
+      <c r="M13" s="98"/>
+      <c r="N13" s="98"/>
+      <c r="O13" s="99"/>
       <c r="P13" s="72"/>
       <c r="Q13" s="73"/>
     </row>
@@ -16230,8 +16232,8 @@
         <v>15</v>
       </c>
       <c r="C14" s="65"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="103"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="101"/>
       <c r="F14" s="64"/>
       <c r="G14" s="68"/>
       <c r="H14" s="69"/>
@@ -16239,9 +16241,9 @@
       <c r="J14" s="64"/>
       <c r="K14" s="64"/>
       <c r="L14" s="71"/>
-      <c r="M14" s="100"/>
-      <c r="N14" s="100"/>
-      <c r="O14" s="101"/>
+      <c r="M14" s="98"/>
+      <c r="N14" s="98"/>
+      <c r="O14" s="99"/>
       <c r="P14" s="72"/>
       <c r="Q14" s="73"/>
     </row>
@@ -16254,8 +16256,8 @@
         <v>16</v>
       </c>
       <c r="C15" s="65"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="103"/>
+      <c r="D15" s="97"/>
+      <c r="E15" s="101"/>
       <c r="F15" s="64"/>
       <c r="G15" s="68"/>
       <c r="H15" s="69"/>
@@ -16263,9 +16265,9 @@
       <c r="J15" s="64"/>
       <c r="K15" s="64"/>
       <c r="L15" s="71"/>
-      <c r="M15" s="100"/>
-      <c r="N15" s="100"/>
-      <c r="O15" s="101"/>
+      <c r="M15" s="98"/>
+      <c r="N15" s="98"/>
+      <c r="O15" s="99"/>
       <c r="P15" s="72"/>
       <c r="Q15" s="73"/>
     </row>
@@ -16279,7 +16281,7 @@
       </c>
       <c r="C16" s="65"/>
       <c r="D16" s="66"/>
-      <c r="E16" s="103"/>
+      <c r="E16" s="101"/>
       <c r="F16" s="64"/>
       <c r="G16" s="68"/>
       <c r="H16" s="69"/>
@@ -16287,9 +16289,9 @@
       <c r="J16" s="64"/>
       <c r="K16" s="64"/>
       <c r="L16" s="71"/>
-      <c r="M16" s="100"/>
-      <c r="N16" s="100"/>
-      <c r="O16" s="101"/>
+      <c r="M16" s="98"/>
+      <c r="N16" s="98"/>
+      <c r="O16" s="99"/>
       <c r="P16" s="72"/>
       <c r="Q16" s="73"/>
     </row>
@@ -16302,8 +16304,8 @@
         <v>18</v>
       </c>
       <c r="C17" s="65"/>
-      <c r="D17" s="99"/>
-      <c r="E17" s="103"/>
+      <c r="D17" s="97"/>
+      <c r="E17" s="101"/>
       <c r="F17" s="64"/>
       <c r="G17" s="68"/>
       <c r="H17" s="69"/>
@@ -16311,9 +16313,9 @@
       <c r="J17" s="64"/>
       <c r="K17" s="64"/>
       <c r="L17" s="71"/>
-      <c r="M17" s="100"/>
-      <c r="N17" s="100"/>
-      <c r="O17" s="101"/>
+      <c r="M17" s="98"/>
+      <c r="N17" s="98"/>
+      <c r="O17" s="99"/>
       <c r="P17" s="72"/>
       <c r="Q17" s="73"/>
     </row>
@@ -16326,8 +16328,8 @@
         <v>19</v>
       </c>
       <c r="C18" s="65"/>
-      <c r="D18" s="99"/>
-      <c r="E18" s="103"/>
+      <c r="D18" s="97"/>
+      <c r="E18" s="101"/>
       <c r="F18" s="64"/>
       <c r="G18" s="68"/>
       <c r="H18" s="69"/>
@@ -16335,9 +16337,9 @@
       <c r="J18" s="64"/>
       <c r="K18" s="64"/>
       <c r="L18" s="71"/>
-      <c r="M18" s="100"/>
-      <c r="N18" s="100"/>
-      <c r="O18" s="101"/>
+      <c r="M18" s="98"/>
+      <c r="N18" s="98"/>
+      <c r="O18" s="99"/>
       <c r="P18" s="72"/>
       <c r="Q18" s="73"/>
     </row>
@@ -16350,8 +16352,8 @@
         <v>20</v>
       </c>
       <c r="C19" s="65"/>
-      <c r="D19" s="99"/>
-      <c r="E19" s="103"/>
+      <c r="D19" s="97"/>
+      <c r="E19" s="101"/>
       <c r="F19" s="64"/>
       <c r="G19" s="68"/>
       <c r="H19" s="69"/>
@@ -16359,9 +16361,9 @@
       <c r="J19" s="64"/>
       <c r="K19" s="64"/>
       <c r="L19" s="71"/>
-      <c r="M19" s="100"/>
-      <c r="N19" s="100"/>
-      <c r="O19" s="102"/>
+      <c r="M19" s="98"/>
+      <c r="N19" s="98"/>
+      <c r="O19" s="100"/>
       <c r="P19" s="75"/>
       <c r="Q19" s="76"/>
     </row>
@@ -16374,8 +16376,8 @@
         <v>21</v>
       </c>
       <c r="C20" s="65"/>
-      <c r="D20" s="99"/>
-      <c r="E20" s="103"/>
+      <c r="D20" s="97"/>
+      <c r="E20" s="101"/>
       <c r="F20" s="64"/>
       <c r="G20" s="68"/>
       <c r="H20" s="69"/>
@@ -16383,9 +16385,9 @@
       <c r="J20" s="64"/>
       <c r="K20" s="64"/>
       <c r="L20" s="71"/>
-      <c r="M20" s="100"/>
-      <c r="N20" s="100"/>
-      <c r="O20" s="102"/>
+      <c r="M20" s="98"/>
+      <c r="N20" s="98"/>
+      <c r="O20" s="100"/>
       <c r="P20" s="75"/>
       <c r="Q20" s="76"/>
     </row>
@@ -16398,8 +16400,8 @@
         <v>24</v>
       </c>
       <c r="C21" s="65"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="103"/>
+      <c r="D21" s="97"/>
+      <c r="E21" s="101"/>
       <c r="F21" s="64"/>
       <c r="G21" s="68"/>
       <c r="H21" s="69"/>
@@ -16407,9 +16409,9 @@
       <c r="J21" s="64"/>
       <c r="K21" s="64"/>
       <c r="L21" s="71"/>
-      <c r="M21" s="100"/>
-      <c r="N21" s="100"/>
-      <c r="O21" s="102"/>
+      <c r="M21" s="98"/>
+      <c r="N21" s="98"/>
+      <c r="O21" s="100"/>
       <c r="P21" s="75"/>
       <c r="Q21" s="76"/>
     </row>
@@ -16423,7 +16425,7 @@
       </c>
       <c r="C22" s="65"/>
       <c r="D22" s="66"/>
-      <c r="E22" s="103"/>
+      <c r="E22" s="101"/>
       <c r="F22" s="64"/>
       <c r="G22" s="68"/>
       <c r="H22" s="69"/>
@@ -16431,9 +16433,9 @@
       <c r="J22" s="64"/>
       <c r="K22" s="64"/>
       <c r="L22" s="71"/>
-      <c r="M22" s="100"/>
-      <c r="N22" s="100"/>
-      <c r="O22" s="102"/>
+      <c r="M22" s="98"/>
+      <c r="N22" s="98"/>
+      <c r="O22" s="100"/>
       <c r="P22" s="75"/>
       <c r="Q22" s="76"/>
     </row>
@@ -16447,7 +16449,7 @@
       </c>
       <c r="C23" s="65"/>
       <c r="D23" s="66"/>
-      <c r="E23" s="103"/>
+      <c r="E23" s="101"/>
       <c r="F23" s="64"/>
       <c r="G23" s="68"/>
       <c r="H23" s="69"/>
@@ -16455,9 +16457,9 @@
       <c r="J23" s="64"/>
       <c r="K23" s="64"/>
       <c r="L23" s="71"/>
-      <c r="M23" s="100"/>
-      <c r="N23" s="100"/>
-      <c r="O23" s="102"/>
+      <c r="M23" s="98"/>
+      <c r="N23" s="98"/>
+      <c r="O23" s="100"/>
       <c r="P23" s="75"/>
       <c r="Q23" s="73"/>
     </row>
@@ -16470,8 +16472,8 @@
         <v>27</v>
       </c>
       <c r="C24" s="65"/>
-      <c r="D24" s="99"/>
-      <c r="E24" s="103"/>
+      <c r="D24" s="97"/>
+      <c r="E24" s="101"/>
       <c r="F24" s="64"/>
       <c r="G24" s="68"/>
       <c r="H24" s="69"/>
@@ -16479,9 +16481,9 @@
       <c r="J24" s="64"/>
       <c r="K24" s="64"/>
       <c r="L24" s="71"/>
-      <c r="M24" s="100"/>
-      <c r="N24" s="100"/>
-      <c r="O24" s="101"/>
+      <c r="M24" s="98"/>
+      <c r="N24" s="98"/>
+      <c r="O24" s="99"/>
       <c r="P24" s="72"/>
       <c r="Q24" s="73"/>
     </row>

</xml_diff>